<commit_message>
First attempt of grouping implemented, second attempt file added to .gitignore
</commit_message>
<xml_diff>
--- a/0-assets/raw_data/main/3-grouping/quarterly_statistics.xlsx
+++ b/0-assets/raw_data/main/3-grouping/quarterly_statistics.xlsx
@@ -465,7 +465,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2006-Q2</t>
+          <t>2010-Q1</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -478,13 +478,13 @@
         <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H2" t="n">
         <v>0</v>
@@ -496,7 +496,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2006-Q3</t>
+          <t>2010-Q2</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -509,13 +509,13 @@
         <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F3" t="n">
         <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H3" t="n">
         <v>0</v>
@@ -527,7 +527,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2006-Q4</t>
+          <t>2010-Q3</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -537,28 +537,28 @@
         <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F4" t="n">
         <v>0</v>
       </c>
       <c r="G4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H4" t="n">
         <v>0</v>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2007-Q1</t>
+          <t>2010-Q4</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -568,16 +568,16 @@
         <v>0</v>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F5" t="n">
         <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H5" t="n">
         <v>0</v>
@@ -589,7 +589,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2007-Q2</t>
+          <t>2011-Q1</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -602,25 +602,25 @@
         <v>0</v>
       </c>
       <c r="E6" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F6" t="n">
         <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H6" t="n">
         <v>0</v>
       </c>
       <c r="I6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2007-Q3</t>
+          <t>2011-Q2</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -630,16 +630,16 @@
         <v>0</v>
       </c>
       <c r="D7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E7" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="F7" t="n">
         <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H7" t="n">
         <v>0</v>
@@ -651,7 +651,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2007-Q4</t>
+          <t>2011-Q3</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -661,10 +661,10 @@
         <v>0</v>
       </c>
       <c r="D8" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="E8" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="F8" t="n">
         <v>0</v>
@@ -676,13 +676,13 @@
         <v>0</v>
       </c>
       <c r="I8" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2008-Q1</t>
+          <t>2011-Q4</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -692,28 +692,28 @@
         <v>0</v>
       </c>
       <c r="D9" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="E9" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="F9" t="n">
         <v>0</v>
       </c>
       <c r="G9" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H9" t="n">
         <v>0</v>
       </c>
       <c r="I9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2008-Q2</t>
+          <t>2012-Q1</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -723,47 +723,47 @@
         <v>0</v>
       </c>
       <c r="D10" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E10" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="F10" t="n">
         <v>0</v>
       </c>
       <c r="G10" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="H10" t="n">
         <v>0</v>
       </c>
       <c r="I10" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2008-Q3</t>
+          <t>2012-Q2</t>
         </is>
       </c>
       <c r="B11" t="n">
         <v>0</v>
       </c>
       <c r="C11" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D11" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="E11" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="F11" t="n">
         <v>0</v>
       </c>
       <c r="G11" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H11" t="n">
         <v>0</v>
@@ -775,153 +775,153 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2008-Q4</t>
+          <t>2012-Q3</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C12" t="n">
         <v>0</v>
       </c>
       <c r="D12" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="E12" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="F12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G12" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H12" t="n">
         <v>0</v>
       </c>
       <c r="I12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2009-Q1</t>
+          <t>2012-Q4</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D13" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="E13" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="F13" t="n">
         <v>0</v>
       </c>
       <c r="G13" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="H13" t="n">
         <v>0</v>
       </c>
       <c r="I13" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2009-Q2</t>
+          <t>2013-Q1</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D14" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="E14" t="n">
-        <v>0</v>
+        <v>44</v>
       </c>
       <c r="F14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G14" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H14" t="n">
         <v>0</v>
       </c>
       <c r="I14" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2009-Q3</t>
+          <t>2013-Q2</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C15" t="n">
         <v>0</v>
       </c>
       <c r="D15" t="n">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="E15" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="F15" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G15" t="n">
         <v>1</v>
       </c>
       <c r="H15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2009-Q4</t>
+          <t>2013-Q3</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C16" t="n">
         <v>0</v>
       </c>
       <c r="D16" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="E16" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="F16" t="n">
         <v>0</v>
       </c>
       <c r="G16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H16" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I16" t="n">
         <v>0</v>
@@ -930,122 +930,122 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2010-Q1</t>
+          <t>2013-Q4</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="C17" t="n">
         <v>0</v>
       </c>
       <c r="D17" t="n">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="E17" t="n">
-        <v>6</v>
+        <v>24</v>
       </c>
       <c r="F17" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H17" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I17" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2010-Q2</t>
+          <t>2014-Q1</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D18" t="n">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="E18" t="n">
-        <v>3</v>
+        <v>24</v>
       </c>
       <c r="F18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G18" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H18" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2010-Q3</t>
+          <t>2014-Q2</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D19" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="E19" t="n">
-        <v>4</v>
+        <v>48</v>
       </c>
       <c r="F19" t="n">
         <v>0</v>
       </c>
       <c r="G19" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2010-Q4</t>
+          <t>2014-Q3</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D20" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="E20" t="n">
+        <v>42</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" t="n">
+        <v>8</v>
+      </c>
+      <c r="H20" t="n">
         <v>6</v>
-      </c>
-      <c r="F20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G20" t="n">
-        <v>3</v>
-      </c>
-      <c r="H20" t="n">
-        <v>0</v>
       </c>
       <c r="I20" t="n">
         <v>0</v>
@@ -1054,122 +1054,122 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2011-Q1</t>
+          <t>2014-Q4</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C21" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D21" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="E21" t="n">
-        <v>5</v>
+        <v>56</v>
       </c>
       <c r="F21" t="n">
         <v>0</v>
       </c>
       <c r="G21" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H21" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I21" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2011-Q2</t>
+          <t>2015-Q1</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="C22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D22" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="E22" t="n">
-        <v>14</v>
+        <v>33</v>
       </c>
       <c r="F22" t="n">
         <v>0</v>
       </c>
       <c r="G22" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="H22" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2011-Q3</t>
+          <t>2015-Q2</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D23" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="E23" t="n">
-        <v>18</v>
+        <v>34</v>
       </c>
       <c r="F23" t="n">
         <v>0</v>
       </c>
       <c r="G23" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H23" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I23" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2011-Q4</t>
+          <t>2015-Q3</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D24" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="E24" t="n">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="F24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G24" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H24" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I24" t="n">
         <v>1</v>
@@ -1178,60 +1178,60 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2012-Q1</t>
+          <t>2015-Q4</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C25" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D25" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="E25" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F25" t="n">
         <v>0</v>
       </c>
       <c r="G25" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="H25" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I25" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2012-Q2</t>
+          <t>2016-Q1</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C26" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D26" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="E26" t="n">
-        <v>21</v>
+        <v>35</v>
       </c>
       <c r="F26" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G26" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="H26" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="I26" t="n">
         <v>0</v>
@@ -1240,29 +1240,29 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2012-Q3</t>
+          <t>2016-Q2</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C27" t="n">
         <v>0</v>
       </c>
       <c r="D27" t="n">
-        <v>5</v>
+        <v>19</v>
       </c>
       <c r="E27" t="n">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="F27" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G27" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="H27" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I27" t="n">
         <v>1</v>
@@ -1271,60 +1271,60 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2012-Q4</t>
+          <t>2016-Q3</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C28" t="n">
         <v>1</v>
       </c>
       <c r="D28" t="n">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="E28" t="n">
+        <v>34</v>
+      </c>
+      <c r="F28" t="n">
+        <v>1</v>
+      </c>
+      <c r="G28" t="n">
         <v>18</v>
       </c>
-      <c r="F28" t="n">
-        <v>0</v>
-      </c>
-      <c r="G28" t="n">
-        <v>8</v>
-      </c>
       <c r="H28" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="I28" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2013-Q1</t>
+          <t>2016-Q4</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C29" t="n">
         <v>1</v>
       </c>
       <c r="D29" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E29" t="n">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="F29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G29" t="n">
+        <v>7</v>
+      </c>
+      <c r="H29" t="n">
         <v>5</v>
-      </c>
-      <c r="H29" t="n">
-        <v>0</v>
       </c>
       <c r="I29" t="n">
         <v>3</v>
@@ -1333,100 +1333,100 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2013-Q2</t>
+          <t>2017-Q1</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C30" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D30" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="E30" t="n">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="F30" t="n">
         <v>1</v>
       </c>
       <c r="G30" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="H30" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="I30" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2013-Q3</t>
+          <t>2017-Q2</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C31" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D31" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E31" t="n">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="F31" t="n">
         <v>0</v>
       </c>
       <c r="G31" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="H31" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I31" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2013-Q4</t>
+          <t>2017-Q3</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="C32" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D32" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="E32" t="n">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="F32" t="n">
         <v>0</v>
       </c>
       <c r="G32" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H32" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="I32" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2014-Q1</t>
+          <t>2017-Q4</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1436,28 +1436,28 @@
         <v>0</v>
       </c>
       <c r="D33" t="n">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="E33" t="n">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="F33" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G33" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="H33" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="I33" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2014-Q2</t>
+          <t>2018-Q1</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -1467,298 +1467,298 @@
         <v>1</v>
       </c>
       <c r="D34" t="n">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="E34" t="n">
-        <v>45</v>
+        <v>22</v>
       </c>
       <c r="F34" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G34" t="n">
-        <v>1</v>
+        <v>28</v>
       </c>
       <c r="H34" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="I34" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2014-Q3</t>
+          <t>2018-Q2</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C35" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D35" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E35" t="n">
-        <v>40</v>
+        <v>29</v>
       </c>
       <c r="F35" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G35" t="n">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="H35" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I35" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2014-Q4</t>
+          <t>2018-Q3</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C36" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D36" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E36" t="n">
-        <v>54</v>
+        <v>25</v>
       </c>
       <c r="F36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G36" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="H36" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="I36" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2015-Q1</t>
+          <t>2018-Q4</t>
         </is>
       </c>
       <c r="B37" t="n">
+        <v>6</v>
+      </c>
+      <c r="C37" t="n">
+        <v>3</v>
+      </c>
+      <c r="D37" t="n">
+        <v>32</v>
+      </c>
+      <c r="E37" t="n">
+        <v>32</v>
+      </c>
+      <c r="F37" t="n">
+        <v>2</v>
+      </c>
+      <c r="G37" t="n">
+        <v>13</v>
+      </c>
+      <c r="H37" t="n">
+        <v>6</v>
+      </c>
+      <c r="I37" t="n">
         <v>5</v>
-      </c>
-      <c r="C37" t="n">
-        <v>1</v>
-      </c>
-      <c r="D37" t="n">
-        <v>12</v>
-      </c>
-      <c r="E37" t="n">
-        <v>27</v>
-      </c>
-      <c r="F37" t="n">
-        <v>0</v>
-      </c>
-      <c r="G37" t="n">
-        <v>6</v>
-      </c>
-      <c r="H37" t="n">
-        <v>0</v>
-      </c>
-      <c r="I37" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2015-Q2</t>
+          <t>2019-Q1</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C38" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D38" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="E38" t="n">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="F38" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G38" t="n">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="H38" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I38" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2015-Q3</t>
+          <t>2019-Q2</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="C39" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="D39" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="E39" t="n">
-        <v>27</v>
+        <v>37</v>
       </c>
       <c r="F39" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G39" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="H39" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I39" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2015-Q4</t>
+          <t>2019-Q3</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>3</v>
+        <v>24</v>
       </c>
       <c r="C40" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D40" t="n">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="E40" t="n">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="F40" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G40" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="H40" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I40" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2016-Q1</t>
+          <t>2019-Q4</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C41" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="D41" t="n">
-        <v>9</v>
+        <v>75</v>
       </c>
       <c r="E41" t="n">
-        <v>31</v>
+        <v>60</v>
       </c>
       <c r="F41" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="G41" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="H41" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="I41" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2016-Q2</t>
+          <t>2020-Q1</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>2</v>
+        <v>38</v>
       </c>
       <c r="C42" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="D42" t="n">
-        <v>5</v>
+        <v>68</v>
       </c>
       <c r="E42" t="n">
-        <v>23</v>
+        <v>38</v>
       </c>
       <c r="F42" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G42" t="n">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="H42" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I42" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2016-Q3</t>
+          <t>2020-Q2</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>2</v>
+        <v>29</v>
       </c>
       <c r="C43" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="D43" t="n">
-        <v>9</v>
+        <v>42</v>
       </c>
       <c r="E43" t="n">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="F43" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G43" t="n">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="H43" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I43" t="n">
         <v>3</v>
@@ -1767,621 +1767,156 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2016-Q4</t>
+          <t>2020-Q3</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="C44" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="D44" t="n">
-        <v>4</v>
+        <v>51</v>
       </c>
       <c r="E44" t="n">
-        <v>29</v>
+        <v>56</v>
       </c>
       <c r="F44" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G44" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H44" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I44" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2017-Q1</t>
+          <t>2020-Q4</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>1</v>
+        <v>31</v>
       </c>
       <c r="C45" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="D45" t="n">
-        <v>11</v>
+        <v>49</v>
       </c>
       <c r="E45" t="n">
-        <v>21</v>
+        <v>34</v>
       </c>
       <c r="F45" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G45" t="n">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="H45" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I45" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2017-Q2</t>
+          <t>2021-Q1</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>1</v>
+        <v>17</v>
       </c>
       <c r="C46" t="n">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="D46" t="n">
-        <v>6</v>
+        <v>54</v>
       </c>
       <c r="E46" t="n">
-        <v>22</v>
+        <v>56</v>
       </c>
       <c r="F46" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="G46" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="H46" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I46" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2017-Q3</t>
+          <t>2021-Q2</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="C47" t="n">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="D47" t="n">
-        <v>10</v>
+        <v>46</v>
       </c>
       <c r="E47" t="n">
-        <v>13</v>
+        <v>57</v>
       </c>
       <c r="F47" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G47" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H47" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I47" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2017-Q4</t>
+          <t>2021-Q3</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>2</v>
+        <v>28</v>
       </c>
       <c r="C48" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="D48" t="n">
-        <v>9</v>
+        <v>46</v>
       </c>
       <c r="E48" t="n">
-        <v>21</v>
+        <v>48</v>
       </c>
       <c r="F48" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G48" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="H48" t="n">
         <v>3</v>
       </c>
       <c r="I48" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>2018-Q1</t>
-        </is>
-      </c>
-      <c r="B49" t="n">
-        <v>0</v>
-      </c>
-      <c r="C49" t="n">
-        <v>1</v>
-      </c>
-      <c r="D49" t="n">
-        <v>4</v>
-      </c>
-      <c r="E49" t="n">
-        <v>19</v>
-      </c>
-      <c r="F49" t="n">
-        <v>1</v>
-      </c>
-      <c r="G49" t="n">
-        <v>28</v>
-      </c>
-      <c r="H49" t="n">
-        <v>4</v>
-      </c>
-      <c r="I49" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>2018-Q2</t>
-        </is>
-      </c>
-      <c r="B50" t="n">
-        <v>2</v>
-      </c>
-      <c r="C50" t="n">
-        <v>1</v>
-      </c>
-      <c r="D50" t="n">
-        <v>6</v>
-      </c>
-      <c r="E50" t="n">
-        <v>22</v>
-      </c>
-      <c r="F50" t="n">
-        <v>1</v>
-      </c>
-      <c r="G50" t="n">
-        <v>16</v>
-      </c>
-      <c r="H50" t="n">
-        <v>4</v>
-      </c>
-      <c r="I50" t="n">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>2018-Q3</t>
-        </is>
-      </c>
-      <c r="B51" t="n">
-        <v>2</v>
-      </c>
-      <c r="C51" t="n">
-        <v>2</v>
-      </c>
-      <c r="D51" t="n">
-        <v>6</v>
-      </c>
-      <c r="E51" t="n">
-        <v>16</v>
-      </c>
-      <c r="F51" t="n">
-        <v>1</v>
-      </c>
-      <c r="G51" t="n">
-        <v>8</v>
-      </c>
-      <c r="H51" t="n">
         <v>5</v>
-      </c>
-      <c r="I51" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>2018-Q4</t>
-        </is>
-      </c>
-      <c r="B52" t="n">
-        <v>3</v>
-      </c>
-      <c r="C52" t="n">
-        <v>2</v>
-      </c>
-      <c r="D52" t="n">
-        <v>15</v>
-      </c>
-      <c r="E52" t="n">
-        <v>19</v>
-      </c>
-      <c r="F52" t="n">
-        <v>2</v>
-      </c>
-      <c r="G52" t="n">
-        <v>13</v>
-      </c>
-      <c r="H52" t="n">
-        <v>3</v>
-      </c>
-      <c r="I52" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>2019-Q1</t>
-        </is>
-      </c>
-      <c r="B53" t="n">
-        <v>6</v>
-      </c>
-      <c r="C53" t="n">
-        <v>2</v>
-      </c>
-      <c r="D53" t="n">
-        <v>9</v>
-      </c>
-      <c r="E53" t="n">
-        <v>20</v>
-      </c>
-      <c r="F53" t="n">
-        <v>1</v>
-      </c>
-      <c r="G53" t="n">
-        <v>17</v>
-      </c>
-      <c r="H53" t="n">
-        <v>0</v>
-      </c>
-      <c r="I53" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>2019-Q2</t>
-        </is>
-      </c>
-      <c r="B54" t="n">
-        <v>11</v>
-      </c>
-      <c r="C54" t="n">
-        <v>2</v>
-      </c>
-      <c r="D54" t="n">
-        <v>13</v>
-      </c>
-      <c r="E54" t="n">
-        <v>26</v>
-      </c>
-      <c r="F54" t="n">
-        <v>0</v>
-      </c>
-      <c r="G54" t="n">
-        <v>8</v>
-      </c>
-      <c r="H54" t="n">
-        <v>3</v>
-      </c>
-      <c r="I54" t="n">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>2019-Q3</t>
-        </is>
-      </c>
-      <c r="B55" t="n">
-        <v>20</v>
-      </c>
-      <c r="C55" t="n">
-        <v>2</v>
-      </c>
-      <c r="D55" t="n">
-        <v>7</v>
-      </c>
-      <c r="E55" t="n">
-        <v>19</v>
-      </c>
-      <c r="F55" t="n">
-        <v>0</v>
-      </c>
-      <c r="G55" t="n">
-        <v>7</v>
-      </c>
-      <c r="H55" t="n">
-        <v>3</v>
-      </c>
-      <c r="I55" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>2019-Q4</t>
-        </is>
-      </c>
-      <c r="B56" t="n">
-        <v>7</v>
-      </c>
-      <c r="C56" t="n">
-        <v>3</v>
-      </c>
-      <c r="D56" t="n">
-        <v>30</v>
-      </c>
-      <c r="E56" t="n">
-        <v>22</v>
-      </c>
-      <c r="F56" t="n">
-        <v>2</v>
-      </c>
-      <c r="G56" t="n">
-        <v>9</v>
-      </c>
-      <c r="H56" t="n">
-        <v>9</v>
-      </c>
-      <c r="I56" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>2020-Q1</t>
-        </is>
-      </c>
-      <c r="B57" t="n">
-        <v>7</v>
-      </c>
-      <c r="C57" t="n">
-        <v>7</v>
-      </c>
-      <c r="D57" t="n">
-        <v>36</v>
-      </c>
-      <c r="E57" t="n">
-        <v>17</v>
-      </c>
-      <c r="F57" t="n">
-        <v>1</v>
-      </c>
-      <c r="G57" t="n">
-        <v>9</v>
-      </c>
-      <c r="H57" t="n">
-        <v>2</v>
-      </c>
-      <c r="I57" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>2020-Q2</t>
-        </is>
-      </c>
-      <c r="B58" t="n">
-        <v>15</v>
-      </c>
-      <c r="C58" t="n">
-        <v>3</v>
-      </c>
-      <c r="D58" t="n">
-        <v>18</v>
-      </c>
-      <c r="E58" t="n">
-        <v>16</v>
-      </c>
-      <c r="F58" t="n">
-        <v>4</v>
-      </c>
-      <c r="G58" t="n">
-        <v>7</v>
-      </c>
-      <c r="H58" t="n">
-        <v>0</v>
-      </c>
-      <c r="I58" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>2020-Q3</t>
-        </is>
-      </c>
-      <c r="B59" t="n">
-        <v>4</v>
-      </c>
-      <c r="C59" t="n">
-        <v>4</v>
-      </c>
-      <c r="D59" t="n">
-        <v>22</v>
-      </c>
-      <c r="E59" t="n">
-        <v>23</v>
-      </c>
-      <c r="F59" t="n">
-        <v>2</v>
-      </c>
-      <c r="G59" t="n">
-        <v>6</v>
-      </c>
-      <c r="H59" t="n">
-        <v>0</v>
-      </c>
-      <c r="I59" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>2020-Q4</t>
-        </is>
-      </c>
-      <c r="B60" t="n">
-        <v>14</v>
-      </c>
-      <c r="C60" t="n">
-        <v>3</v>
-      </c>
-      <c r="D60" t="n">
-        <v>27</v>
-      </c>
-      <c r="E60" t="n">
-        <v>11</v>
-      </c>
-      <c r="F60" t="n">
-        <v>3</v>
-      </c>
-      <c r="G60" t="n">
-        <v>8</v>
-      </c>
-      <c r="H60" t="n">
-        <v>1</v>
-      </c>
-      <c r="I60" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>2021-Q1</t>
-        </is>
-      </c>
-      <c r="B61" t="n">
-        <v>9</v>
-      </c>
-      <c r="C61" t="n">
-        <v>5</v>
-      </c>
-      <c r="D61" t="n">
-        <v>28</v>
-      </c>
-      <c r="E61" t="n">
-        <v>25</v>
-      </c>
-      <c r="F61" t="n">
-        <v>3</v>
-      </c>
-      <c r="G61" t="n">
-        <v>4</v>
-      </c>
-      <c r="H61" t="n">
-        <v>3</v>
-      </c>
-      <c r="I61" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>2021-Q2</t>
-        </is>
-      </c>
-      <c r="B62" t="n">
-        <v>9</v>
-      </c>
-      <c r="C62" t="n">
-        <v>5</v>
-      </c>
-      <c r="D62" t="n">
-        <v>22</v>
-      </c>
-      <c r="E62" t="n">
-        <v>34</v>
-      </c>
-      <c r="F62" t="n">
-        <v>1</v>
-      </c>
-      <c r="G62" t="n">
-        <v>6</v>
-      </c>
-      <c r="H62" t="n">
-        <v>0</v>
-      </c>
-      <c r="I62" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>2021-Q3</t>
-        </is>
-      </c>
-      <c r="B63" t="n">
-        <v>23</v>
-      </c>
-      <c r="C63" t="n">
-        <v>2</v>
-      </c>
-      <c r="D63" t="n">
-        <v>16</v>
-      </c>
-      <c r="E63" t="n">
-        <v>30</v>
-      </c>
-      <c r="F63" t="n">
-        <v>4</v>
-      </c>
-      <c r="G63" t="n">
-        <v>6</v>
-      </c>
-      <c r="H63" t="n">
-        <v>2</v>
-      </c>
-      <c r="I63" t="n">
-        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Second attempt implemented, flair annotation begun
</commit_message>
<xml_diff>
--- a/0-assets/raw_data/main/3-grouping/quarterly_statistics.xlsx
+++ b/0-assets/raw_data/main/3-grouping/quarterly_statistics.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Quarterly counts" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Run info" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -475,22 +476,22 @@
         <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>88</v>
       </c>
       <c r="E2" t="n">
-        <v>6</v>
+        <v>485</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>1</v>
+        <v>221</v>
       </c>
       <c r="H2" t="n">
         <v>0</v>
       </c>
       <c r="I2" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
     </row>
     <row r="3">
@@ -506,22 +507,22 @@
         <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>163</v>
       </c>
       <c r="E3" t="n">
-        <v>3</v>
+        <v>740</v>
       </c>
       <c r="F3" t="n">
         <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>3</v>
+        <v>270</v>
       </c>
       <c r="H3" t="n">
         <v>0</v>
       </c>
       <c r="I3" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4">
@@ -537,22 +538,22 @@
         <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>1</v>
+        <v>342</v>
       </c>
       <c r="E4" t="n">
-        <v>4</v>
+        <v>1282</v>
       </c>
       <c r="F4" t="n">
         <v>0</v>
       </c>
       <c r="G4" t="n">
-        <v>2</v>
+        <v>293</v>
       </c>
       <c r="H4" t="n">
         <v>0</v>
       </c>
       <c r="I4" t="n">
-        <v>1</v>
+        <v>42</v>
       </c>
     </row>
     <row r="5">
@@ -565,25 +566,25 @@
         <v>0</v>
       </c>
       <c r="C5" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D5" t="n">
-        <v>4</v>
+        <v>493</v>
       </c>
       <c r="E5" t="n">
-        <v>6</v>
+        <v>1442</v>
       </c>
       <c r="F5" t="n">
         <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v>3</v>
+        <v>384</v>
       </c>
       <c r="H5" t="n">
         <v>0</v>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>97</v>
       </c>
     </row>
     <row r="6">
@@ -596,25 +597,25 @@
         <v>0</v>
       </c>
       <c r="C6" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>656</v>
       </c>
       <c r="E6" t="n">
-        <v>6</v>
+        <v>1816</v>
       </c>
       <c r="F6" t="n">
         <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>2</v>
+        <v>505</v>
       </c>
       <c r="H6" t="n">
         <v>0</v>
       </c>
       <c r="I6" t="n">
-        <v>2</v>
+        <v>122</v>
       </c>
     </row>
     <row r="7">
@@ -627,25 +628,25 @@
         <v>0</v>
       </c>
       <c r="C7" t="n">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="D7" t="n">
-        <v>2</v>
+        <v>772</v>
       </c>
       <c r="E7" t="n">
-        <v>14</v>
+        <v>2276</v>
       </c>
       <c r="F7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G7" t="n">
-        <v>2</v>
+        <v>611</v>
       </c>
       <c r="H7" t="n">
         <v>0</v>
       </c>
       <c r="I7" t="n">
-        <v>0</v>
+        <v>105</v>
       </c>
     </row>
     <row r="8">
@@ -655,28 +656,28 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C8" t="n">
-        <v>0</v>
+        <v>44</v>
       </c>
       <c r="D8" t="n">
-        <v>7</v>
+        <v>1365</v>
       </c>
       <c r="E8" t="n">
-        <v>19</v>
+        <v>2848</v>
       </c>
       <c r="F8" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="G8" t="n">
-        <v>1</v>
+        <v>519</v>
       </c>
       <c r="H8" t="n">
         <v>0</v>
       </c>
       <c r="I8" t="n">
-        <v>3</v>
+        <v>196</v>
       </c>
     </row>
     <row r="9">
@@ -686,28 +687,28 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0</v>
+        <v>112</v>
       </c>
       <c r="C9" t="n">
-        <v>0</v>
+        <v>68</v>
       </c>
       <c r="D9" t="n">
-        <v>9</v>
+        <v>1538</v>
       </c>
       <c r="E9" t="n">
-        <v>15</v>
+        <v>3222</v>
       </c>
       <c r="F9" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="G9" t="n">
-        <v>6</v>
+        <v>766</v>
       </c>
       <c r="H9" t="n">
         <v>0</v>
       </c>
       <c r="I9" t="n">
-        <v>1</v>
+        <v>230</v>
       </c>
     </row>
     <row r="10">
@@ -717,28 +718,28 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0</v>
+        <v>144</v>
       </c>
       <c r="C10" t="n">
-        <v>0</v>
+        <v>94</v>
       </c>
       <c r="D10" t="n">
-        <v>5</v>
+        <v>2343</v>
       </c>
       <c r="E10" t="n">
-        <v>24</v>
+        <v>3678</v>
       </c>
       <c r="F10" t="n">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="G10" t="n">
-        <v>9</v>
+        <v>833</v>
       </c>
       <c r="H10" t="n">
         <v>0</v>
       </c>
       <c r="I10" t="n">
-        <v>2</v>
+        <v>312</v>
       </c>
     </row>
     <row r="11">
@@ -748,28 +749,28 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0</v>
+        <v>259</v>
       </c>
       <c r="C11" t="n">
-        <v>2</v>
+        <v>99</v>
       </c>
       <c r="D11" t="n">
-        <v>10</v>
+        <v>3573</v>
       </c>
       <c r="E11" t="n">
-        <v>22</v>
+        <v>4473</v>
       </c>
       <c r="F11" t="n">
-        <v>0</v>
+        <v>51</v>
       </c>
       <c r="G11" t="n">
-        <v>3</v>
+        <v>875</v>
       </c>
       <c r="H11" t="n">
         <v>0</v>
       </c>
       <c r="I11" t="n">
-        <v>0</v>
+        <v>218</v>
       </c>
     </row>
     <row r="12">
@@ -779,28 +780,28 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1</v>
+        <v>518</v>
       </c>
       <c r="C12" t="n">
-        <v>0</v>
+        <v>115</v>
       </c>
       <c r="D12" t="n">
-        <v>24</v>
+        <v>4861</v>
       </c>
       <c r="E12" t="n">
-        <v>23</v>
+        <v>5804</v>
       </c>
       <c r="F12" t="n">
-        <v>1</v>
+        <v>122</v>
       </c>
       <c r="G12" t="n">
-        <v>3</v>
+        <v>979</v>
       </c>
       <c r="H12" t="n">
         <v>0</v>
       </c>
       <c r="I12" t="n">
-        <v>1</v>
+        <v>209</v>
       </c>
     </row>
     <row r="13">
@@ -810,28 +811,28 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>4</v>
+        <v>789</v>
       </c>
       <c r="C13" t="n">
-        <v>1</v>
+        <v>97</v>
       </c>
       <c r="D13" t="n">
-        <v>30</v>
+        <v>6582</v>
       </c>
       <c r="E13" t="n">
-        <v>21</v>
+        <v>5947</v>
       </c>
       <c r="F13" t="n">
-        <v>0</v>
+        <v>157</v>
       </c>
       <c r="G13" t="n">
-        <v>8</v>
+        <v>792</v>
       </c>
       <c r="H13" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I13" t="n">
-        <v>3</v>
+        <v>206</v>
       </c>
     </row>
     <row r="14">
@@ -841,28 +842,28 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>3</v>
+        <v>940</v>
       </c>
       <c r="C14" t="n">
-        <v>1</v>
+        <v>195</v>
       </c>
       <c r="D14" t="n">
-        <v>30</v>
+        <v>7494</v>
       </c>
       <c r="E14" t="n">
-        <v>44</v>
+        <v>6801</v>
       </c>
       <c r="F14" t="n">
-        <v>1</v>
+        <v>52</v>
       </c>
       <c r="G14" t="n">
-        <v>5</v>
+        <v>586</v>
       </c>
       <c r="H14" t="n">
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="I14" t="n">
-        <v>3</v>
+        <v>209</v>
       </c>
     </row>
     <row r="15">
@@ -872,28 +873,28 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1</v>
+        <v>1130</v>
       </c>
       <c r="C15" t="n">
-        <v>0</v>
+        <v>132</v>
       </c>
       <c r="D15" t="n">
-        <v>32</v>
+        <v>8283</v>
       </c>
       <c r="E15" t="n">
-        <v>16</v>
+        <v>6141</v>
       </c>
       <c r="F15" t="n">
-        <v>2</v>
+        <v>44</v>
       </c>
       <c r="G15" t="n">
-        <v>1</v>
+        <v>568</v>
       </c>
       <c r="H15" t="n">
-        <v>1</v>
+        <v>243</v>
       </c>
       <c r="I15" t="n">
-        <v>1</v>
+        <v>165</v>
       </c>
     </row>
     <row r="16">
@@ -903,28 +904,28 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>3</v>
+        <v>3451</v>
       </c>
       <c r="C16" t="n">
-        <v>0</v>
+        <v>114</v>
       </c>
       <c r="D16" t="n">
-        <v>30</v>
+        <v>8786</v>
       </c>
       <c r="E16" t="n">
-        <v>24</v>
+        <v>5452</v>
       </c>
       <c r="F16" t="n">
-        <v>0</v>
+        <v>48</v>
       </c>
       <c r="G16" t="n">
-        <v>3</v>
+        <v>413</v>
       </c>
       <c r="H16" t="n">
-        <v>2</v>
+        <v>268</v>
       </c>
       <c r="I16" t="n">
-        <v>0</v>
+        <v>165</v>
       </c>
     </row>
     <row r="17">
@@ -934,28 +935,28 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>7</v>
+        <v>5439</v>
       </c>
       <c r="C17" t="n">
-        <v>0</v>
+        <v>185</v>
       </c>
       <c r="D17" t="n">
-        <v>26</v>
+        <v>9771</v>
       </c>
       <c r="E17" t="n">
-        <v>24</v>
+        <v>5686</v>
       </c>
       <c r="F17" t="n">
-        <v>2</v>
+        <v>81</v>
       </c>
       <c r="G17" t="n">
-        <v>2</v>
+        <v>333</v>
       </c>
       <c r="H17" t="n">
-        <v>3</v>
+        <v>422</v>
       </c>
       <c r="I17" t="n">
-        <v>2</v>
+        <v>174</v>
       </c>
     </row>
     <row r="18">
@@ -965,28 +966,28 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>3</v>
+        <v>5222</v>
       </c>
       <c r="C18" t="n">
-        <v>1</v>
+        <v>219</v>
       </c>
       <c r="D18" t="n">
-        <v>26</v>
+        <v>10209</v>
       </c>
       <c r="E18" t="n">
-        <v>24</v>
+        <v>6227</v>
       </c>
       <c r="F18" t="n">
-        <v>1</v>
+        <v>53</v>
       </c>
       <c r="G18" t="n">
-        <v>1</v>
+        <v>340</v>
       </c>
       <c r="H18" t="n">
-        <v>4</v>
+        <v>694</v>
       </c>
       <c r="I18" t="n">
-        <v>1</v>
+        <v>189</v>
       </c>
     </row>
     <row r="19">
@@ -996,28 +997,28 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>2</v>
+        <v>4346</v>
       </c>
       <c r="C19" t="n">
-        <v>1</v>
+        <v>164</v>
       </c>
       <c r="D19" t="n">
-        <v>25</v>
+        <v>9733</v>
       </c>
       <c r="E19" t="n">
-        <v>48</v>
+        <v>10912</v>
       </c>
       <c r="F19" t="n">
-        <v>0</v>
+        <v>42</v>
       </c>
       <c r="G19" t="n">
-        <v>1</v>
+        <v>275</v>
       </c>
       <c r="H19" t="n">
-        <v>1</v>
+        <v>651</v>
       </c>
       <c r="I19" t="n">
-        <v>0</v>
+        <v>152</v>
       </c>
     </row>
     <row r="20">
@@ -1027,28 +1028,28 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>3</v>
+        <v>4213</v>
       </c>
       <c r="C20" t="n">
-        <v>1</v>
+        <v>196</v>
       </c>
       <c r="D20" t="n">
-        <v>30</v>
+        <v>8962</v>
       </c>
       <c r="E20" t="n">
-        <v>42</v>
+        <v>12294</v>
       </c>
       <c r="F20" t="n">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="G20" t="n">
-        <v>8</v>
+        <v>282</v>
       </c>
       <c r="H20" t="n">
-        <v>6</v>
+        <v>959</v>
       </c>
       <c r="I20" t="n">
-        <v>0</v>
+        <v>201</v>
       </c>
     </row>
     <row r="21">
@@ -1058,28 +1059,28 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>2</v>
+        <v>2458</v>
       </c>
       <c r="C21" t="n">
-        <v>2</v>
+        <v>243</v>
       </c>
       <c r="D21" t="n">
-        <v>22</v>
+        <v>7886</v>
       </c>
       <c r="E21" t="n">
-        <v>56</v>
+        <v>12815</v>
       </c>
       <c r="F21" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="G21" t="n">
-        <v>0</v>
+        <v>302</v>
       </c>
       <c r="H21" t="n">
-        <v>4</v>
+        <v>926</v>
       </c>
       <c r="I21" t="n">
-        <v>0</v>
+        <v>200</v>
       </c>
     </row>
     <row r="22">
@@ -1089,28 +1090,28 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>5</v>
+        <v>2411</v>
       </c>
       <c r="C22" t="n">
-        <v>1</v>
+        <v>282</v>
       </c>
       <c r="D22" t="n">
-        <v>24</v>
+        <v>7775</v>
       </c>
       <c r="E22" t="n">
-        <v>33</v>
+        <v>9524</v>
       </c>
       <c r="F22" t="n">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="G22" t="n">
-        <v>6</v>
+        <v>261</v>
       </c>
       <c r="H22" t="n">
-        <v>3</v>
+        <v>956</v>
       </c>
       <c r="I22" t="n">
-        <v>1</v>
+        <v>284</v>
       </c>
     </row>
     <row r="23">
@@ -1120,28 +1121,28 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>4</v>
+        <v>1790</v>
       </c>
       <c r="C23" t="n">
-        <v>1</v>
+        <v>295</v>
       </c>
       <c r="D23" t="n">
+        <v>7533</v>
+      </c>
+      <c r="E23" t="n">
+        <v>9392</v>
+      </c>
+      <c r="F23" t="n">
         <v>30</v>
       </c>
-      <c r="E23" t="n">
-        <v>34</v>
-      </c>
-      <c r="F23" t="n">
-        <v>0</v>
-      </c>
       <c r="G23" t="n">
-        <v>4</v>
+        <v>457</v>
       </c>
       <c r="H23" t="n">
-        <v>5</v>
+        <v>1061</v>
       </c>
       <c r="I23" t="n">
-        <v>2</v>
+        <v>277</v>
       </c>
     </row>
     <row r="24">
@@ -1151,28 +1152,28 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>2</v>
+        <v>1797</v>
       </c>
       <c r="C24" t="n">
-        <v>1</v>
+        <v>297</v>
       </c>
       <c r="D24" t="n">
-        <v>25</v>
+        <v>8119</v>
       </c>
       <c r="E24" t="n">
-        <v>29</v>
+        <v>9028</v>
       </c>
       <c r="F24" t="n">
-        <v>1</v>
+        <v>52</v>
       </c>
       <c r="G24" t="n">
-        <v>7</v>
+        <v>1013</v>
       </c>
       <c r="H24" t="n">
-        <v>5</v>
+        <v>1097</v>
       </c>
       <c r="I24" t="n">
-        <v>1</v>
+        <v>435</v>
       </c>
     </row>
     <row r="25">
@@ -1182,28 +1183,28 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>4</v>
+        <v>1466</v>
       </c>
       <c r="C25" t="n">
-        <v>3</v>
+        <v>282</v>
       </c>
       <c r="D25" t="n">
-        <v>22</v>
+        <v>7344</v>
       </c>
       <c r="E25" t="n">
-        <v>23</v>
+        <v>9354</v>
       </c>
       <c r="F25" t="n">
-        <v>0</v>
+        <v>52</v>
       </c>
       <c r="G25" t="n">
-        <v>5</v>
+        <v>1282</v>
       </c>
       <c r="H25" t="n">
-        <v>4</v>
+        <v>1000</v>
       </c>
       <c r="I25" t="n">
-        <v>1</v>
+        <v>417</v>
       </c>
     </row>
     <row r="26">
@@ -1213,28 +1214,28 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>1</v>
+        <v>1444</v>
       </c>
       <c r="C26" t="n">
-        <v>1</v>
+        <v>383</v>
       </c>
       <c r="D26" t="n">
-        <v>30</v>
+        <v>8141</v>
       </c>
       <c r="E26" t="n">
-        <v>35</v>
+        <v>8597</v>
       </c>
       <c r="F26" t="n">
-        <v>2</v>
+        <v>149</v>
       </c>
       <c r="G26" t="n">
-        <v>8</v>
+        <v>3106</v>
       </c>
       <c r="H26" t="n">
-        <v>6</v>
+        <v>985</v>
       </c>
       <c r="I26" t="n">
-        <v>0</v>
+        <v>480</v>
       </c>
     </row>
     <row r="27">
@@ -1244,28 +1245,28 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>2</v>
+        <v>1358</v>
       </c>
       <c r="C27" t="n">
-        <v>0</v>
+        <v>372</v>
       </c>
       <c r="D27" t="n">
-        <v>19</v>
+        <v>7123</v>
       </c>
       <c r="E27" t="n">
-        <v>24</v>
+        <v>7724</v>
       </c>
       <c r="F27" t="n">
-        <v>3</v>
+        <v>142</v>
       </c>
       <c r="G27" t="n">
-        <v>7</v>
+        <v>2658</v>
       </c>
       <c r="H27" t="n">
-        <v>3</v>
+        <v>867</v>
       </c>
       <c r="I27" t="n">
-        <v>1</v>
+        <v>473</v>
       </c>
     </row>
     <row r="28">
@@ -1275,28 +1276,28 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>2</v>
+        <v>1928</v>
       </c>
       <c r="C28" t="n">
-        <v>1</v>
+        <v>388</v>
       </c>
       <c r="D28" t="n">
-        <v>27</v>
+        <v>6944</v>
       </c>
       <c r="E28" t="n">
-        <v>34</v>
+        <v>8543</v>
       </c>
       <c r="F28" t="n">
-        <v>1</v>
+        <v>192</v>
       </c>
       <c r="G28" t="n">
-        <v>18</v>
+        <v>1784</v>
       </c>
       <c r="H28" t="n">
-        <v>7</v>
+        <v>1010</v>
       </c>
       <c r="I28" t="n">
-        <v>3</v>
+        <v>479</v>
       </c>
     </row>
     <row r="29">
@@ -1306,28 +1307,28 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>0</v>
+        <v>1277</v>
       </c>
       <c r="C29" t="n">
-        <v>1</v>
+        <v>399</v>
       </c>
       <c r="D29" t="n">
-        <v>12</v>
+        <v>7681</v>
       </c>
       <c r="E29" t="n">
-        <v>32</v>
+        <v>8306</v>
       </c>
       <c r="F29" t="n">
-        <v>1</v>
+        <v>287</v>
       </c>
       <c r="G29" t="n">
-        <v>7</v>
+        <v>2321</v>
       </c>
       <c r="H29" t="n">
-        <v>5</v>
+        <v>1050</v>
       </c>
       <c r="I29" t="n">
-        <v>3</v>
+        <v>612</v>
       </c>
     </row>
     <row r="30">
@@ -1337,28 +1338,28 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>2</v>
+        <v>1583</v>
       </c>
       <c r="C30" t="n">
-        <v>2</v>
+        <v>397</v>
       </c>
       <c r="D30" t="n">
-        <v>24</v>
+        <v>7460</v>
       </c>
       <c r="E30" t="n">
-        <v>24</v>
+        <v>7700</v>
       </c>
       <c r="F30" t="n">
-        <v>1</v>
+        <v>642</v>
       </c>
       <c r="G30" t="n">
-        <v>14</v>
+        <v>2429</v>
       </c>
       <c r="H30" t="n">
-        <v>8</v>
+        <v>1171</v>
       </c>
       <c r="I30" t="n">
-        <v>0</v>
+        <v>596</v>
       </c>
     </row>
     <row r="31">
@@ -1368,28 +1369,28 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>2</v>
+        <v>1071</v>
       </c>
       <c r="C31" t="n">
-        <v>3</v>
+        <v>428</v>
       </c>
       <c r="D31" t="n">
-        <v>14</v>
+        <v>7633</v>
       </c>
       <c r="E31" t="n">
-        <v>25</v>
+        <v>7737</v>
       </c>
       <c r="F31" t="n">
-        <v>0</v>
+        <v>245</v>
       </c>
       <c r="G31" t="n">
-        <v>8</v>
+        <v>2318</v>
       </c>
       <c r="H31" t="n">
-        <v>3</v>
+        <v>1161</v>
       </c>
       <c r="I31" t="n">
-        <v>3</v>
+        <v>793</v>
       </c>
     </row>
     <row r="32">
@@ -1399,28 +1400,28 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>3</v>
+        <v>970</v>
       </c>
       <c r="C32" t="n">
-        <v>2</v>
+        <v>381</v>
       </c>
       <c r="D32" t="n">
-        <v>24</v>
+        <v>7116</v>
       </c>
       <c r="E32" t="n">
-        <v>14</v>
+        <v>6903</v>
       </c>
       <c r="F32" t="n">
-        <v>0</v>
+        <v>164</v>
       </c>
       <c r="G32" t="n">
-        <v>4</v>
+        <v>2415</v>
       </c>
       <c r="H32" t="n">
-        <v>6</v>
+        <v>1200</v>
       </c>
       <c r="I32" t="n">
-        <v>5</v>
+        <v>823</v>
       </c>
     </row>
     <row r="33">
@@ -1430,28 +1431,28 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>2</v>
+        <v>975</v>
       </c>
       <c r="C33" t="n">
-        <v>0</v>
+        <v>448</v>
       </c>
       <c r="D33" t="n">
-        <v>23</v>
+        <v>7652</v>
       </c>
       <c r="E33" t="n">
-        <v>26</v>
+        <v>6840</v>
       </c>
       <c r="F33" t="n">
-        <v>0</v>
+        <v>117</v>
       </c>
       <c r="G33" t="n">
-        <v>11</v>
+        <v>2689</v>
       </c>
       <c r="H33" t="n">
-        <v>9</v>
+        <v>1292</v>
       </c>
       <c r="I33" t="n">
-        <v>3</v>
+        <v>866</v>
       </c>
     </row>
     <row r="34">
@@ -1461,28 +1462,28 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>2</v>
+        <v>1047</v>
       </c>
       <c r="C34" t="n">
-        <v>1</v>
+        <v>558</v>
       </c>
       <c r="D34" t="n">
-        <v>12</v>
+        <v>7111</v>
       </c>
       <c r="E34" t="n">
-        <v>22</v>
+        <v>7307</v>
       </c>
       <c r="F34" t="n">
-        <v>3</v>
+        <v>250</v>
       </c>
       <c r="G34" t="n">
-        <v>28</v>
+        <v>3039</v>
       </c>
       <c r="H34" t="n">
-        <v>8</v>
+        <v>1102</v>
       </c>
       <c r="I34" t="n">
-        <v>5</v>
+        <v>879</v>
       </c>
     </row>
     <row r="35">
@@ -1492,28 +1493,28 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>4</v>
+        <v>1022</v>
       </c>
       <c r="C35" t="n">
-        <v>2</v>
+        <v>750</v>
       </c>
       <c r="D35" t="n">
-        <v>21</v>
+        <v>7774</v>
       </c>
       <c r="E35" t="n">
-        <v>29</v>
+        <v>8630</v>
       </c>
       <c r="F35" t="n">
-        <v>3</v>
+        <v>455</v>
       </c>
       <c r="G35" t="n">
-        <v>17</v>
+        <v>3151</v>
       </c>
       <c r="H35" t="n">
-        <v>10</v>
+        <v>1497</v>
       </c>
       <c r="I35" t="n">
-        <v>10</v>
+        <v>997</v>
       </c>
     </row>
     <row r="36">
@@ -1523,28 +1524,28 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>2</v>
+        <v>1426</v>
       </c>
       <c r="C36" t="n">
-        <v>3</v>
+        <v>859</v>
       </c>
       <c r="D36" t="n">
-        <v>16</v>
+        <v>7946</v>
       </c>
       <c r="E36" t="n">
-        <v>25</v>
+        <v>8489</v>
       </c>
       <c r="F36" t="n">
-        <v>1</v>
+        <v>504</v>
       </c>
       <c r="G36" t="n">
-        <v>8</v>
+        <v>3876</v>
       </c>
       <c r="H36" t="n">
-        <v>8</v>
+        <v>1619</v>
       </c>
       <c r="I36" t="n">
-        <v>5</v>
+        <v>1015</v>
       </c>
     </row>
     <row r="37">
@@ -1554,28 +1555,28 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>6</v>
+        <v>1975</v>
       </c>
       <c r="C37" t="n">
-        <v>3</v>
+        <v>1156</v>
       </c>
       <c r="D37" t="n">
-        <v>32</v>
+        <v>8761</v>
       </c>
       <c r="E37" t="n">
-        <v>32</v>
+        <v>8794</v>
       </c>
       <c r="F37" t="n">
-        <v>2</v>
+        <v>509</v>
       </c>
       <c r="G37" t="n">
-        <v>13</v>
+        <v>3500</v>
       </c>
       <c r="H37" t="n">
-        <v>6</v>
+        <v>1383</v>
       </c>
       <c r="I37" t="n">
-        <v>5</v>
+        <v>939</v>
       </c>
     </row>
     <row r="38">
@@ -1585,28 +1586,28 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>6</v>
+        <v>3647</v>
       </c>
       <c r="C38" t="n">
-        <v>2</v>
+        <v>1311</v>
       </c>
       <c r="D38" t="n">
-        <v>20</v>
+        <v>9823</v>
       </c>
       <c r="E38" t="n">
-        <v>37</v>
+        <v>10303</v>
       </c>
       <c r="F38" t="n">
-        <v>2</v>
+        <v>461</v>
       </c>
       <c r="G38" t="n">
-        <v>17</v>
+        <v>3542</v>
       </c>
       <c r="H38" t="n">
-        <v>1</v>
+        <v>1391</v>
       </c>
       <c r="I38" t="n">
-        <v>7</v>
+        <v>998</v>
       </c>
     </row>
     <row r="39">
@@ -1616,28 +1617,28 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>11</v>
+        <v>5990</v>
       </c>
       <c r="C39" t="n">
-        <v>6</v>
+        <v>1156</v>
       </c>
       <c r="D39" t="n">
-        <v>30</v>
+        <v>9013</v>
       </c>
       <c r="E39" t="n">
-        <v>37</v>
+        <v>11713</v>
       </c>
       <c r="F39" t="n">
-        <v>0</v>
+        <v>369</v>
       </c>
       <c r="G39" t="n">
-        <v>9</v>
+        <v>2497</v>
       </c>
       <c r="H39" t="n">
-        <v>5</v>
+        <v>1569</v>
       </c>
       <c r="I39" t="n">
-        <v>7</v>
+        <v>902</v>
       </c>
     </row>
     <row r="40">
@@ -1647,28 +1648,28 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>24</v>
+        <v>7112</v>
       </c>
       <c r="C40" t="n">
-        <v>5</v>
+        <v>1230</v>
       </c>
       <c r="D40" t="n">
-        <v>22</v>
+        <v>9892</v>
       </c>
       <c r="E40" t="n">
-        <v>26</v>
+        <v>12211</v>
       </c>
       <c r="F40" t="n">
-        <v>1</v>
+        <v>447</v>
       </c>
       <c r="G40" t="n">
-        <v>7</v>
+        <v>2869</v>
       </c>
       <c r="H40" t="n">
-        <v>3</v>
+        <v>1559</v>
       </c>
       <c r="I40" t="n">
-        <v>4</v>
+        <v>1085</v>
       </c>
     </row>
     <row r="41">
@@ -1678,28 +1679,28 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>30</v>
+        <v>5972</v>
       </c>
       <c r="C41" t="n">
-        <v>10</v>
+        <v>1529</v>
       </c>
       <c r="D41" t="n">
-        <v>75</v>
+        <v>9558</v>
       </c>
       <c r="E41" t="n">
-        <v>60</v>
+        <v>11661</v>
       </c>
       <c r="F41" t="n">
-        <v>6</v>
+        <v>505</v>
       </c>
       <c r="G41" t="n">
-        <v>10</v>
+        <v>2739</v>
       </c>
       <c r="H41" t="n">
-        <v>13</v>
+        <v>1482</v>
       </c>
       <c r="I41" t="n">
-        <v>4</v>
+        <v>1237</v>
       </c>
     </row>
     <row r="42">
@@ -1709,28 +1710,28 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>38</v>
+        <v>5321</v>
       </c>
       <c r="C42" t="n">
-        <v>12</v>
+        <v>1605</v>
       </c>
       <c r="D42" t="n">
-        <v>68</v>
+        <v>9023</v>
       </c>
       <c r="E42" t="n">
-        <v>38</v>
+        <v>12437</v>
       </c>
       <c r="F42" t="n">
-        <v>2</v>
+        <v>550</v>
       </c>
       <c r="G42" t="n">
-        <v>15</v>
+        <v>2978</v>
       </c>
       <c r="H42" t="n">
-        <v>4</v>
+        <v>1164</v>
       </c>
       <c r="I42" t="n">
-        <v>6</v>
+        <v>1204</v>
       </c>
     </row>
     <row r="43">
@@ -1740,28 +1741,28 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>29</v>
+        <v>6935</v>
       </c>
       <c r="C43" t="n">
-        <v>8</v>
+        <v>1822</v>
       </c>
       <c r="D43" t="n">
-        <v>42</v>
+        <v>9724</v>
       </c>
       <c r="E43" t="n">
-        <v>32</v>
+        <v>13045</v>
       </c>
       <c r="F43" t="n">
-        <v>4</v>
+        <v>944</v>
       </c>
       <c r="G43" t="n">
-        <v>7</v>
+        <v>2236</v>
       </c>
       <c r="H43" t="n">
-        <v>4</v>
+        <v>641</v>
       </c>
       <c r="I43" t="n">
-        <v>3</v>
+        <v>1067</v>
       </c>
     </row>
     <row r="44">
@@ -1771,28 +1772,28 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>21</v>
+        <v>6637</v>
       </c>
       <c r="C44" t="n">
-        <v>11</v>
+        <v>2315</v>
       </c>
       <c r="D44" t="n">
-        <v>51</v>
+        <v>11449</v>
       </c>
       <c r="E44" t="n">
-        <v>56</v>
+        <v>12412</v>
       </c>
       <c r="F44" t="n">
-        <v>3</v>
+        <v>987</v>
       </c>
       <c r="G44" t="n">
-        <v>6</v>
+        <v>2268</v>
       </c>
       <c r="H44" t="n">
-        <v>0</v>
+        <v>500</v>
       </c>
       <c r="I44" t="n">
-        <v>3</v>
+        <v>1214</v>
       </c>
     </row>
     <row r="45">
@@ -1802,28 +1803,28 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>31</v>
+        <v>5002</v>
       </c>
       <c r="C45" t="n">
-        <v>13</v>
+        <v>2334</v>
       </c>
       <c r="D45" t="n">
-        <v>49</v>
+        <v>9801</v>
       </c>
       <c r="E45" t="n">
-        <v>34</v>
+        <v>10560</v>
       </c>
       <c r="F45" t="n">
-        <v>5</v>
+        <v>1077</v>
       </c>
       <c r="G45" t="n">
-        <v>8</v>
+        <v>2854</v>
       </c>
       <c r="H45" t="n">
-        <v>5</v>
+        <v>442</v>
       </c>
       <c r="I45" t="n">
-        <v>2</v>
+        <v>956</v>
       </c>
     </row>
     <row r="46">
@@ -1833,28 +1834,28 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>17</v>
+        <v>4626</v>
       </c>
       <c r="C46" t="n">
-        <v>15</v>
+        <v>2510</v>
       </c>
       <c r="D46" t="n">
-        <v>54</v>
+        <v>10640</v>
       </c>
       <c r="E46" t="n">
-        <v>56</v>
+        <v>13212</v>
       </c>
       <c r="F46" t="n">
-        <v>7</v>
+        <v>660</v>
       </c>
       <c r="G46" t="n">
-        <v>4</v>
+        <v>2276</v>
       </c>
       <c r="H46" t="n">
-        <v>3</v>
+        <v>363</v>
       </c>
       <c r="I46" t="n">
-        <v>8</v>
+        <v>1148</v>
       </c>
     </row>
     <row r="47">
@@ -1864,28 +1865,28 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>10</v>
+        <v>5582</v>
       </c>
       <c r="C47" t="n">
-        <v>16</v>
+        <v>3109</v>
       </c>
       <c r="D47" t="n">
-        <v>46</v>
+        <v>12673</v>
       </c>
       <c r="E47" t="n">
-        <v>57</v>
+        <v>14624</v>
       </c>
       <c r="F47" t="n">
-        <v>6</v>
+        <v>504</v>
       </c>
       <c r="G47" t="n">
-        <v>6</v>
+        <v>1641</v>
       </c>
       <c r="H47" t="n">
-        <v>0</v>
+        <v>309</v>
       </c>
       <c r="I47" t="n">
-        <v>5</v>
+        <v>1304</v>
       </c>
     </row>
     <row r="48">
@@ -1895,28 +1896,113 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>28</v>
+        <v>6765</v>
       </c>
       <c r="C48" t="n">
-        <v>9</v>
+        <v>3479</v>
       </c>
       <c r="D48" t="n">
-        <v>46</v>
+        <v>14478</v>
       </c>
       <c r="E48" t="n">
-        <v>48</v>
+        <v>17377</v>
       </c>
       <c r="F48" t="n">
-        <v>6</v>
+        <v>447</v>
       </c>
       <c r="G48" t="n">
-        <v>6</v>
+        <v>1579</v>
       </c>
       <c r="H48" t="n">
-        <v>3</v>
+        <v>552</v>
       </c>
       <c r="I48" t="n">
-        <v>5</v>
+        <v>1453</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>run started</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>2026-10-06T12:36:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>input</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>/Users/uni/Documents/GitHub/shadow_moses/0-assets/raw_data/main/2-filtering/filtered_comments.jsonl</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>comments processed</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>53,006,559</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>input pass</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>0h 07m 15s</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>xlsx writing</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>0h 03m 00s</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>total runtime</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>0h 10m 16s</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>